<commit_message>
feat: add physical push button — GPIO 5, ISR debounce, toggle pump
Hardware:
- Bouton poussoir étanche IP67 sur GPIO 5 (INPUT_PULLUP)
- Ajouté à BOM (bouton métal 12mm, ~2.50€)
- Ajouté à pin_assignment.md

Firmware:
- ISR FALLING avec debounce 300ms (IRAM_ATTR)
- Pompe OFF + appui → start cycle (durée config, failsafes actifs)
- Pompe ON + appui → stop immédiat
- Failsafe actif + appui → 3 blinks LED (feedback erreur)
- Fonctionne dans tous les modes, même sans WiFi
- Alerte Telegram envoyée sur arrosage manuel

Docs:
- CLAUDE.md mis à jour (pin, comportement, GPIO libres)
- pin_assignment.md mis à jour
</commit_message>
<xml_diff>
--- a/docs/BOM_v3_plug_and_play.xlsx
+++ b/docs/BOM_v3_plug_and_play.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="149">
   <si>
     <t xml:space="preserve">BALCONY HYDRA v3 — BOM Plug-and-Play (Zéro Soudure)</t>
   </si>
@@ -365,6 +365,15 @@
   </si>
   <si>
     <t xml:space="preserve">BOÎTIER &amp; MONTAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bouton poussoir étanche IP67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Momentané NO, câble pré-serti, montage panel 12mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress (bouton métal LED 12mm)</t>
   </si>
   <si>
     <t xml:space="preserve">Boîtier étanche IP65 ABS</t>
@@ -464,9 +473,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -635,7 +645,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -645,6 +655,20 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
@@ -676,11 +700,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -693,7 +721,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -701,39 +729,63 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -741,11 +793,11 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -753,7 +805,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -761,19 +813,23 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1029,1470 +1085,1506 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="35"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="10" t="n">
         <f aca="false">E6*F6</f>
         <v>25</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="10" t="n">
         <f aca="false">E7*F7</f>
         <v>30</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <f aca="false">E8*F8</f>
         <v>18</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <f aca="false">E9*F9</f>
         <v>5</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="12" t="n">
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="13" t="n">
         <f aca="false">SUM(G6:G9)</f>
         <v>78</v>
       </c>
-      <c r="H10" s="13"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="n">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="10" t="n">
         <f aca="false">E12*F12</f>
         <v>5</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="10" t="n">
         <f aca="false">E13*F13</f>
         <v>8</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="10" t="n">
         <f aca="false">E14*F14</f>
         <v>5</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="9" t="n">
         <v>3.5</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" s="10" t="n">
         <f aca="false">E15*F15</f>
         <v>3.5</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="10" t="n">
         <f aca="false">E16*F16</f>
         <v>2</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="10" t="n">
         <f aca="false">E17*F17</f>
         <v>0.2</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="10" t="n">
         <f aca="false">E18*F18</f>
         <v>0.2</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="9" t="n">
         <v>0.2</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G19" s="10" t="n">
         <f aca="false">E19*F19</f>
         <v>0.4</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="12" t="n">
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="13" t="n">
         <f aca="false">SUM(G12:G19)</f>
         <v>24.3</v>
       </c>
-      <c r="H20" s="13"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="H20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="n">
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="10" t="n">
         <f aca="false">E22*F22</f>
         <v>16</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="H22" s="11" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="9" t="n">
         <v>4.5</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G23" s="10" t="n">
         <f aca="false">E23*F23</f>
         <v>9</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="F24" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G24" s="9" t="n">
+      <c r="G24" s="10" t="n">
         <f aca="false">E24*F24</f>
         <v>2.5</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F25" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="9" t="n">
+      <c r="G25" s="10" t="n">
         <f aca="false">E25*F25</f>
         <v>2</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="12" t="n">
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="13" t="n">
         <f aca="false">SUM(G22:G25)</f>
         <v>29.5</v>
       </c>
-      <c r="H26" s="13"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="H26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="n">
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="F28" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="9" t="n">
+      <c r="G28" s="10" t="n">
         <f aca="false">E28*F28</f>
         <v>0</v>
       </c>
-      <c r="H28" s="10" t="s">
+      <c r="H28" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="F29" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="G29" s="9" t="n">
+      <c r="G29" s="10" t="n">
         <f aca="false">E29*F29</f>
         <v>12</v>
       </c>
-      <c r="H29" s="10" t="s">
+      <c r="H29" s="11" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="8" t="n">
+      <c r="F30" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="G30" s="9" t="n">
+      <c r="G30" s="10" t="n">
         <f aca="false">E30*F30</f>
         <v>6</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" s="11" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="E31" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="F31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G31" s="9" t="n">
+      <c r="G31" s="10" t="n">
         <f aca="false">E31*F31</f>
         <v>6</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" s="11" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="E32" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F32" s="8" t="n">
+      <c r="F32" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G32" s="9" t="n">
+      <c r="G32" s="10" t="n">
         <f aca="false">E32*F32</f>
         <v>3</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="H32" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E33" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F33" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G33" s="9" t="n">
+      <c r="G33" s="10" t="n">
         <f aca="false">E33*F33</f>
         <v>10</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="H33" s="11" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="E34" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="9" t="n">
         <v>0.4</v>
       </c>
-      <c r="G34" s="9" t="n">
+      <c r="G34" s="10" t="n">
         <f aca="false">E34*F34</f>
         <v>8</v>
       </c>
-      <c r="H34" s="10" t="s">
+      <c r="H34" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="9" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="9" t="n">
+      <c r="G35" s="10" t="n">
         <f aca="false">E35*F35</f>
         <v>4</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="H35" s="11" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E36" s="5" t="n">
+      <c r="E36" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F36" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G36" s="9" t="n">
+      <c r="G36" s="10" t="n">
         <f aca="false">E36*F36</f>
         <v>3</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="H36" s="11" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="12" t="n">
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="13" t="n">
         <f aca="false">SUM(G28:G36)</f>
         <v>52</v>
       </c>
-      <c r="H37" s="13"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
+      <c r="H37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="n">
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="E39" s="5" t="n">
+      <c r="E39" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F39" s="8" t="n">
+      <c r="F39" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="G39" s="9" t="n">
+      <c r="G39" s="10" t="n">
         <f aca="false">E39*F39</f>
         <v>5</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="H39" s="11" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="E40" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="9" t="n">
         <v>0.6</v>
       </c>
-      <c r="G40" s="9" t="n">
+      <c r="G40" s="10" t="n">
         <f aca="false">E40*F40</f>
         <v>6</v>
       </c>
-      <c r="H40" s="10" t="s">
+      <c r="H40" s="11" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="n">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="E41" s="5" t="n">
+      <c r="E41" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F41" s="8" t="n">
+      <c r="F41" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="G41" s="9" t="n">
+      <c r="G41" s="10" t="n">
         <f aca="false">E41*F41</f>
         <v>4</v>
       </c>
-      <c r="H41" s="10" t="s">
+      <c r="H41" s="11" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E42" s="5" t="n">
+      <c r="E42" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F42" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G42" s="9" t="n">
+      <c r="G42" s="10" t="n">
         <f aca="false">E42*F42</f>
         <v>4</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H42" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="n">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E43" s="5" t="n">
+      <c r="E43" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F43" s="9" t="n">
         <v>0.05</v>
       </c>
-      <c r="G43" s="9" t="n">
+      <c r="G43" s="10" t="n">
         <f aca="false">E43*F43</f>
         <v>2</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="H43" s="11" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="n">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E44" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F44" s="8" t="n">
+      <c r="F44" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="G44" s="9" t="n">
+      <c r="G44" s="10" t="n">
         <f aca="false">E44*F44</f>
         <v>8</v>
       </c>
-      <c r="H44" s="10" t="s">
+      <c r="H44" s="11" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="n">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D45" s="7" t="s">
+      <c r="D45" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E45" s="5" t="n">
+      <c r="E45" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F45" s="8" t="n">
+      <c r="F45" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G45" s="9" t="n">
+      <c r="G45" s="10" t="n">
         <f aca="false">E45*F45</f>
         <v>3</v>
       </c>
-      <c r="H45" s="10" t="s">
+      <c r="H45" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="n">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E46" s="5" t="n">
+      <c r="E46" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F46" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="9" t="n">
+      <c r="G46" s="10" t="n">
         <f aca="false">E46*F46</f>
         <v>2</v>
       </c>
-      <c r="H46" s="10" t="s">
+      <c r="H46" s="11" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="11" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="12" t="n">
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="13" t="n">
         <f aca="false">SUM(G39:G46)</f>
         <v>34</v>
       </c>
-      <c r="H47" s="13"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="H47" s="14"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B48" s="4"/>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="n">
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="B49" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G49" s="18" t="n">
+        <f aca="false">E49*F49</f>
+        <v>2.5</v>
+      </c>
+      <c r="H49" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B50" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C49" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E49" s="5" t="n">
+      <c r="C50" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E50" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F49" s="8" t="n">
+      <c r="F50" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="G49" s="9" t="n">
+      <c r="G50" s="10" t="n">
         <f aca="false">E49*F49</f>
+        <v>2.5</v>
+      </c>
+      <c r="H50" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G51" s="10" t="n">
+        <f aca="false">E50*F50</f>
         <v>12</v>
       </c>
-      <c r="H49" s="10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="n">
+      <c r="H51" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G52" s="10" t="n">
+        <f aca="false">E51*F51</f>
+        <v>4</v>
+      </c>
+      <c r="H52" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G53" s="10" t="n">
+        <f aca="false">E52*F52</f>
+        <v>2.4</v>
+      </c>
+      <c r="H53" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B50" s="6" t="s">
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B54" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C50" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E50" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F50" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <f aca="false">E50*F50</f>
-        <v>4</v>
-      </c>
-      <c r="H50" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="B51" s="6" t="s">
+      <c r="C54" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G54" s="10" t="n">
+        <f aca="false">E53*F53</f>
+        <v>1.4</v>
+      </c>
+      <c r="H54" s="11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C51" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E51" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F51" s="8" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <f aca="false">E51*F51</f>
-        <v>2.4</v>
-      </c>
-      <c r="H51" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="B52" s="6" t="s">
+      <c r="C55" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G55" s="10" t="n">
+        <f aca="false">E54*F54</f>
+        <v>2</v>
+      </c>
+      <c r="H55" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B56" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C52" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="E52" s="5" t="n">
+      <c r="C56" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G56" s="10" t="n">
+        <f aca="false">E55*F55</f>
+        <v>3</v>
+      </c>
+      <c r="H56" s="11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E57" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F52" s="8" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G52" s="9" t="n">
-        <f aca="false">E52*F52</f>
-        <v>1.4</v>
-      </c>
-      <c r="H52" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E53" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <f aca="false">E53*F53</f>
-        <v>2</v>
-      </c>
-      <c r="H53" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="5" t="n">
-        <v>39</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D54" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="E54" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="8" t="n">
+      <c r="F57" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G54" s="9" t="n">
-        <f aca="false">E54*F54</f>
-        <v>3</v>
-      </c>
-      <c r="H54" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="B55" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="E55" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="8" t="n">
+      <c r="G57" s="10" t="n">
+        <f aca="false">E56*F56</f>
         <v>2.5</v>
       </c>
-      <c r="G55" s="9" t="n">
-        <f aca="false">E55*F55</f>
-        <v>2.5</v>
-      </c>
-      <c r="H55" s="10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="E56" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F56" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="G56" s="9" t="n">
-        <f aca="false">E56*F56</f>
-        <v>6</v>
-      </c>
-      <c r="H56" s="10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
-      <c r="F57" s="11"/>
-      <c r="G57" s="12" t="n">
+      <c r="H57" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="B58" s="19"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="20"/>
+      <c r="G58" s="13" t="n">
         <f aca="false">SUM(G49:G56)</f>
-        <v>33.3</v>
-      </c>
-      <c r="H57" s="13"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="16" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="H58" s="14"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="21"/>
+      <c r="B59" s="21"/>
+      <c r="C59" s="21"/>
+      <c r="D59" s="21"/>
+      <c r="E59" s="21"/>
+      <c r="F59" s="21"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="B60" s="22"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="23" t="n">
         <f aca="false">G10+G20+G26+G37+G47+G57</f>
-        <v>251.1</v>
-      </c>
-      <c r="H59" s="17"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="18" t="s">
-        <v>136</v>
-      </c>
-      <c r="B60" s="18"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="18"/>
-      <c r="E60" s="18"/>
-      <c r="F60" s="18"/>
-      <c r="G60" s="19" t="n">
+        <v>220.3</v>
+      </c>
+      <c r="H60" s="24"/>
+    </row>
+    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="B61" s="25"/>
+      <c r="C61" s="25"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="26" t="n">
         <f aca="false">G59*0.15</f>
-        <v>37.665</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="B62" s="19"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="28" t="n">
         <f aca="false">G59+G60</f>
-        <v>288.765</v>
-      </c>
-      <c r="H61" s="22"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="23" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-      <c r="G64" s="24"/>
-      <c r="H64" s="24"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="B65" s="24"/>
-      <c r="C65" s="24"/>
-      <c r="D65" s="24"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="24"/>
-      <c r="G65" s="24"/>
-      <c r="H65" s="24"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="24" t="s">
+        <v>220.3</v>
+      </c>
+      <c r="H62" s="29"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="B66" s="24"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="24"/>
-      <c r="F66" s="24"/>
-      <c r="G66" s="24"/>
-      <c r="H66" s="24"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="24" t="s">
+      <c r="B64" s="30"/>
+      <c r="C64" s="30"/>
+      <c r="D64" s="30"/>
+      <c r="E64" s="30"/>
+      <c r="F64" s="30"/>
+      <c r="G64" s="30"/>
+      <c r="H64" s="30"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="B67" s="24"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="24"/>
-      <c r="F67" s="24"/>
-      <c r="G67" s="24"/>
-      <c r="H67" s="24"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="24" t="s">
+      <c r="B65" s="31"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="31"/>
+      <c r="E65" s="31"/>
+      <c r="F65" s="31"/>
+      <c r="G65" s="31"/>
+      <c r="H65" s="31"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="31" t="s">
         <v>143</v>
       </c>
-      <c r="B68" s="24"/>
-      <c r="C68" s="24"/>
-      <c r="D68" s="24"/>
-      <c r="E68" s="24"/>
-      <c r="F68" s="24"/>
-      <c r="G68" s="24"/>
-      <c r="H68" s="24"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="24" t="s">
+      <c r="B66" s="31"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="31"/>
+      <c r="E66" s="31"/>
+      <c r="F66" s="31"/>
+      <c r="G66" s="31"/>
+      <c r="H66" s="31"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="B69" s="24"/>
-      <c r="C69" s="24"/>
-      <c r="D69" s="24"/>
-      <c r="E69" s="24"/>
-      <c r="F69" s="24"/>
-      <c r="G69" s="24"/>
-      <c r="H69" s="24"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="24" t="s">
+      <c r="B67" s="31"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="31"/>
+      <c r="F67" s="31"/>
+      <c r="G67" s="31"/>
+      <c r="H67" s="31"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="B70" s="24"/>
-      <c r="C70" s="24"/>
-      <c r="D70" s="24"/>
-      <c r="E70" s="24"/>
-      <c r="F70" s="24"/>
-      <c r="G70" s="24"/>
-      <c r="H70" s="24"/>
+      <c r="B68" s="31"/>
+      <c r="C68" s="31"/>
+      <c r="D68" s="31"/>
+      <c r="E68" s="31"/>
+      <c r="F68" s="31"/>
+      <c r="G68" s="31"/>
+      <c r="H68" s="31"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="B69" s="31"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="E69" s="31"/>
+      <c r="F69" s="31"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="31"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="31" t="s">
+        <v>147</v>
+      </c>
+      <c r="B70" s="31"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="31"/>
+      <c r="E70" s="31"/>
+      <c r="F70" s="31"/>
+      <c r="G70" s="31"/>
+      <c r="H70" s="31"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="32" t="s">
+        <v>148</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>

<commit_message>
feat: dual enclosure layout + thermal protection + BOM safety components
Physical layout (full sun, no shade, Cogolin):
- Enclosure 1 (ELECTRONICS): white ABS 200×150×85mm, wall-mounted
  ESP32, MUX, MOSFET module, relay, LED RGB, button
- Enclosure 2 (ENERGY): white ABS 250×200×120mm, floor behind water tanks
  Battery LiFePO4, MPPT, LM2596, fuses (5A+3A), thermal fuse 72°C
  Ventilated: 4 stainless grilles (convection) + mosquito mesh
  Reflective: aluminium bubble foil on lid
  Shielded: 3×25L water tanks as thermal mass barrier

BOM additions (9 new items):
- Enclosure 2 (energy, ventilated, white)
- 4× stainless ventilation grilles with insect mesh
- Reflective aluminium bubble insulation
- Inter-enclosure 18AWG cable + Wago
- LED RGB 5mm common cathode
- Relay module 5V opto-isolated
- Fuse 5A + inline holder (battery)
- Fuse 3A + inline holder (pump line)
- Thermal fuse 72°C (battery cable, irreversible)

Safety analysis: ASCII thermal diagram, component-to-enclosure mapping
</commit_message>
<xml_diff>
--- a/docs/BOM_v3_plug_and_play.xlsx
+++ b/docs/BOM_v3_plug_and_play.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="172">
   <si>
     <t xml:space="preserve">BALCONY HYDRA v3 — BOM Plug-and-Play (Zéro Soudure)</t>
   </si>
@@ -94,6 +94,15 @@
     <t xml:space="preserve">Amazon</t>
   </si>
   <si>
+    <t xml:space="preserve">Fusible thermique 72°C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-coupure irréversible si T° batterie &gt;72°C. En série sur câble + batterie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress (thermal fuse 72°C 10A)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sous-total ÉNERGIE &amp; CHARGE</t>
   </si>
   <si>
@@ -166,6 +175,39 @@
     <t xml:space="preserve">Électrolytique, filtrage LM2596</t>
   </si>
   <si>
+    <t xml:space="preserve">MCU &amp; CONNECTIQUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED RGB 5mm common cathode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rouge+Vert+Bleu, 3.3V compatible, diffuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress (lot 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module relais 5V 1 canal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opto-isolé, borniers à vis, NO/NC. Relais sécurité pompe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusible 5A + porte-fusible inline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verre 5×20mm, porte-fusible à vis sur câble batterie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress / Leroy Merlin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusible 3A + porte-fusible inline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verre 5×20mm, sur ligne 12V pompe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sous-total MCU &amp; CONNECTIQUE PLUG-AND-PLA</t>
   </si>
   <si>
@@ -340,9 +382,6 @@
     <t xml:space="preserve">1-2m, pour capteurs humidité déportés</t>
   </si>
   <si>
-    <t xml:space="preserve">AliExpress (lot 10)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Gaine thermorétractable (assortiment)</t>
   </si>
   <si>
@@ -376,10 +415,49 @@
     <t xml:space="preserve">AliExpress (bouton métal LED 12mm)</t>
   </si>
   <si>
-    <t xml:space="preserve">Boîtier étanche IP65 ABS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">200×150×85mm, charnière, vis inox</t>
+    <t xml:space="preserve">Boîtier 1 — Électronique IP65 BLANC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABS blanc 200×150×85mm, charnière, vis inox. ESP32+MUX+relais+LED+bouton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress / Amazon — CHOISIR BLANC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boîtier 2 — Énergie IP65 BLANC ventilé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABS blanc 250×200×120mm, grilles ventilation inox haut+bas. Batterie+MPPT+LM2596+fusibles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress / Amazon — BLANC + percer grilles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grille ventilation inox + moustiquaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40×20mm, inox 304, avec filtre anti-insectes. 2 en bas + 2 en haut (convection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress (lot grilles aération)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isolant réflectif aluminium bulle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feuille alu/bulle, découpe couvercle boîtier énergie. Renvoie rayonnement solaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leroy Merlin / Bricomarché (rouleau camping-car)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Câble liaison inter-boîtiers 12V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silicone 18AWG rouge+noir, 1.5m, avec Wago chaque extrémité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress + Wago 221-412</t>
   </si>
   <si>
     <t xml:space="preserve">Presse-étoupe PG7</t>
@@ -406,9 +484,6 @@
     <t xml:space="preserve">Montage interne boîtier, clip Wago</t>
   </si>
   <si>
-    <t xml:space="preserve">AliExpress / Leroy Merlin</t>
-  </si>
-  <si>
     <t xml:space="preserve">Plaque support perforée</t>
   </si>
   <si>
@@ -422,12 +497,6 @@
   </si>
   <si>
     <t xml:space="preserve">AliExpress (kit assortiment)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gel silicone IP68 (Wago Gelbox)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protection Wago extérieures si exposées</t>
   </si>
   <si>
     <t xml:space="preserve">Amazon / Leroy Merlin</t>
@@ -478,7 +547,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -561,6 +630,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FFE74C3C"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF27AE60"/>
@@ -635,7 +711,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC0392B"/>
-        <bgColor rgb="FF993366"/>
+        <bgColor rgb="FFE74C3C"/>
       </patternFill>
     </fill>
     <fill>
@@ -645,7 +721,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -674,6 +750,13 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -700,7 +783,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -749,10 +832,30 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -761,27 +864,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -789,31 +876,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -821,15 +904,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -865,7 +944,7 @@
       <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFE74C3C"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
@@ -1085,7 +1164,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -1269,65 +1348,65 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="6" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="13" t="n">
+      <c r="D10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <f aca="false">E10*F10</f>
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13" t="n">
         <f aca="false">SUM(G6:G9)</f>
         <v>78</v>
       </c>
-      <c r="H10" s="14"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="H11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="8" t="s">
+      <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G12" s="10" t="n">
-        <f aca="false">E12*F12</f>
-        <v>5</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>29</v>
-      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>30</v>
@@ -1339,11 +1418,11 @@
         <v>1</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G13" s="10" t="n">
-        <f aca="false">E13*F13</f>
-        <v>8</v>
+        <f aca="false">E12*F12</f>
+        <v>0</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>32</v>
@@ -1351,10 +1430,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>33</v>
@@ -1363,13 +1442,13 @@
         <v>34</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G14" s="10" t="n">
-        <f aca="false">E14*F14</f>
+        <f aca="false">E13*F13</f>
         <v>5</v>
       </c>
       <c r="H14" s="11" t="s">
@@ -1378,10 +1457,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>36</v>
@@ -1390,14 +1469,14 @@
         <v>37</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="G15" s="10" t="n">
-        <f aca="false">E15*F15</f>
-        <v>3.5</v>
+        <f aca="false">E14*F14</f>
+        <v>8</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>38</v>
@@ -1405,10 +1484,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>39</v>
@@ -1420,49 +1499,49 @@
         <v>1</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="G16" s="10" t="n">
-        <f aca="false">E16*F16</f>
-        <v>2</v>
+        <f aca="false">E15*F15</f>
+        <v>5</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F17" s="9" t="n">
-        <v>0.1</v>
-      </c>
       <c r="G17" s="10" t="n">
-        <f aca="false">E17*F17</f>
-        <v>0.2</v>
+        <f aca="false">E16*F16</f>
+        <v>3.5</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>44</v>
@@ -1477,1113 +1556,1299 @@
         <v>0.1</v>
       </c>
       <c r="G18" s="10" t="n">
+        <f aca="false">E17*F17</f>
+        <v>2</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G19" s="10" t="n">
         <f aca="false">E18*F18</f>
         <v>0.2</v>
       </c>
-      <c r="H18" s="11" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="n">
+      <c r="H19" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="6" t="n">
+      <c r="B20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F20" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G20" s="10" t="n">
         <f aca="false">E19*F19</f>
+        <v>0.2</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <f aca="false">E20*F20</f>
         <v>0.4</v>
       </c>
-      <c r="H19" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="13" t="n">
-        <f aca="false">SUM(G12:G19)</f>
-        <v>24.3</v>
-      </c>
-      <c r="H20" s="14"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
+      <c r="H21" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="7" t="s">
+        <v>12.2</v>
+      </c>
+      <c r="B22" s="16" t="s">
         <v>51</v>
       </c>
+      <c r="C22" s="16" t="s">
+        <v>55</v>
+      </c>
       <c r="D22" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <f aca="false">E22*F22</f>
-        <v>16</v>
+        <v>1</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <f aca="false">E21*F21</f>
+        <v>0.3</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>54</v>
+        <v>12.3</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>57</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="9" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G23" s="10" t="n">
-        <f aca="false">E23*F23</f>
-        <v>9</v>
+      <c r="G23" s="12" t="n">
+        <f aca="false">E22*F22</f>
+        <v>2</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>56</v>
+        <v>12.4</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>60</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G24" s="10" t="n">
-        <f aca="false">E24*F24</f>
-        <v>2.5</v>
+      <c r="F24" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="12" t="n">
+        <f aca="false">E23*F23</f>
+        <v>2</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="9" t="n">
+      <c r="A25" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="18" t="n">
+        <f aca="false">SUM(G12:G19)</f>
+        <v>23.7</v>
+      </c>
+      <c r="H25" s="19"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="15"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <f aca="false">E22*F22</f>
         <v>2</v>
       </c>
-      <c r="G25" s="10" t="n">
-        <f aca="false">E25*F25</f>
-        <v>2</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="13" t="n">
-        <f aca="false">SUM(G22:G25)</f>
-        <v>29.5</v>
-      </c>
-      <c r="H26" s="14"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
+      <c r="H27" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G28" s="10" t="n">
-        <f aca="false">E28*F28</f>
-        <v>0</v>
+        <f aca="false">E23*F23</f>
+        <v>2</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>12</v>
+        <v>2.5</v>
       </c>
       <c r="G29" s="10" t="n">
-        <f aca="false">E29*F29</f>
-        <v>12</v>
+        <f aca="false">E24*F24</f>
+        <v>2</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G30" s="10" t="n">
-        <f aca="false">E30*F30</f>
-        <v>6</v>
+        <f aca="false">E25*F25</f>
+        <v>0</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G31" s="10" t="n">
-        <f aca="false">E31*F31</f>
-        <v>6</v>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>71</v>
-      </c>
+      <c r="A31" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="18" t="n">
+        <f aca="false">SUM(G22:G25)</f>
+        <v>28</v>
+      </c>
+      <c r="H31" s="19"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" s="8" t="s">
+      <c r="A32" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G32" s="10" t="n">
-        <f aca="false">E32*F32</f>
-        <v>3</v>
-      </c>
-      <c r="H32" s="11" t="s">
-        <v>76</v>
-      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C33" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>77</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>78</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" s="9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G33" s="10" t="n">
-        <f aca="false">E33*F33</f>
-        <v>10</v>
+        <f aca="false">E28*F28</f>
+        <v>9</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>0.4</v>
+        <v>12</v>
       </c>
       <c r="G34" s="10" t="n">
-        <f aca="false">E34*F34</f>
-        <v>8</v>
+        <f aca="false">E29*F29</f>
+        <v>2.5</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="F35" s="9" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="G35" s="10" t="n">
-        <f aca="false">E35*F35</f>
-        <v>4</v>
+        <f aca="false">E30*F30</f>
+        <v>2</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C36" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <f aca="false">E31*F31</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="F36" s="9" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G36" s="10" t="n">
-        <f aca="false">E36*F36</f>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H36" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="13" t="n">
-        <f aca="false">SUM(G28:G36)</f>
-        <v>52</v>
-      </c>
-      <c r="H37" s="14"/>
+      <c r="G37" s="10" t="n">
+        <f aca="false">E32*F32</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
+      <c r="A38" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <f aca="false">E33*F33</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="10" t="n">
-        <f aca="false">E39*F39</f>
-        <v>5</v>
+        <f aca="false">E34*F34</f>
+        <v>12</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="G40" s="10" t="n">
-        <f aca="false">E40*F40</f>
+        <f aca="false">E35*F35</f>
         <v>6</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="G41" s="10" t="n">
-        <f aca="false">E41*F41</f>
-        <v>4</v>
+        <f aca="false">E36*F36</f>
+        <v>6</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="G42" s="10" t="n">
-        <f aca="false">E42*F42</f>
-        <v>4</v>
-      </c>
-      <c r="H42" s="11" t="s">
-        <v>35</v>
-      </c>
+      <c r="A42" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="18" t="n">
+        <f aca="false">SUM(G28:G36)</f>
+        <v>45.5</v>
+      </c>
+      <c r="H42" s="19"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="F43" s="9" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G43" s="10" t="n">
-        <f aca="false">E43*F43</f>
-        <v>2</v>
-      </c>
-      <c r="H43" s="11" t="s">
+      <c r="A43" s="5" t="s">
         <v>103</v>
       </c>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="15"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E44" s="6" t="n">
         <v>10</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G44" s="10" t="n">
-        <f aca="false">E44*F44</f>
+        <f aca="false">E39*F39</f>
         <v>8</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C45" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G45" s="10" t="n">
+        <f aca="false">E40*F40</f>
+        <v>4</v>
+      </c>
+      <c r="H45" s="11" t="s">
         <v>107</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="E45" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G45" s="10" t="n">
-        <f aca="false">E45*F45</f>
-        <v>3</v>
-      </c>
-      <c r="H45" s="11" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="G46" s="10" t="n">
-        <f aca="false">E46*F46</f>
-        <v>2</v>
+        <f aca="false">E41*F41</f>
+        <v>3</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="13" t="n">
-        <f aca="false">SUM(G39:G46)</f>
-        <v>34</v>
-      </c>
-      <c r="H47" s="14"/>
+      <c r="A47" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G47" s="10" t="n">
+        <f aca="false">E42*F42</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="11" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
+      <c r="A48" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <f aca="false">E43*F43</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="B49" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>115</v>
+        <v>31</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>118</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="17" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G49" s="18" t="n">
-        <f aca="false">E49*F49</f>
-        <v>2.5</v>
+        <v>10</v>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G49" s="10" t="n">
+        <f aca="false">E44*F44</f>
+        <v>5</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>117</v>
+        <v>54</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E50" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="9" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="G50" s="10" t="n">
-        <f aca="false">E49*F49</f>
-        <v>2.5</v>
+        <f aca="false">E45*F45</f>
+        <v>6</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F51" s="9" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="G51" s="10" t="n">
-        <f aca="false">E50*F50</f>
-        <v>12</v>
+        <f aca="false">E46*F46</f>
+        <v>4</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="E52" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G52" s="10" t="n">
-        <f aca="false">E51*F51</f>
-        <v>4</v>
-      </c>
-      <c r="H52" s="11" t="s">
-        <v>106</v>
-      </c>
+      <c r="A52" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="18" t="n">
+        <f aca="false">SUM(G39:G46)</f>
+        <v>84.5</v>
+      </c>
+      <c r="H52" s="19"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="B53" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="E53" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F53" s="9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G53" s="10" t="n">
-        <f aca="false">E52*F52</f>
-        <v>2.4</v>
-      </c>
-      <c r="H53" s="11" t="s">
-        <v>35</v>
-      </c>
+      <c r="A53" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B53" s="14"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="14"/>
+      <c r="G53" s="14"/>
+      <c r="H53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="n">
-        <v>38</v>
+        <v>33.5</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E54" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G54" s="10" t="n">
-        <f aca="false">E53*F53</f>
-        <v>1.4</v>
+        <f aca="false">E49*F49</f>
+        <v>8</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E55" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F55" s="9" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G55" s="10" t="n">
-        <f aca="false">E54*F54</f>
-        <v>2</v>
+        <f aca="false">E49*F49</f>
+        <v>8</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>35</v>
+        <v>133</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>131</v>
+        <v>34.1</v>
+      </c>
+      <c r="B56" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C56" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E56" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F56" s="9" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G56" s="10" t="n">
-        <f aca="false">E55*F55</f>
-        <v>3</v>
+      <c r="F56" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="G56" s="12" t="n">
+        <f aca="false">E51*F51</f>
+        <v>2</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G57" s="12" t="n">
+        <f aca="false">E52*F52</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="B58" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C58" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G58" s="12" t="n">
+        <f aca="false">E53*F53</f>
+        <v>0</v>
+      </c>
+      <c r="H58" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="6" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G59" s="12" t="n">
+        <f aca="false">E54*F54</f>
+        <v>2.5</v>
+      </c>
+      <c r="H59" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G60" s="10" t="n">
+        <f aca="false">E50*F50</f>
+        <v>3</v>
+      </c>
+      <c r="H60" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G61" s="10" t="n">
+        <f aca="false">E51*F51</f>
+        <v>2</v>
+      </c>
+      <c r="H61" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G62" s="10" t="n">
+        <f aca="false">E52*F52</f>
+        <v>0</v>
+      </c>
+      <c r="H62" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G63" s="10" t="n">
+        <f aca="false">E53*F53</f>
+        <v>0</v>
+      </c>
+      <c r="H63" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="E64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G64" s="6" t="n">
+        <f aca="false">E54*F54</f>
+        <v>2.5</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <f aca="false">E55*F55</f>
+        <v>12</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B57" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F57" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G57" s="10" t="n">
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="6" t="n">
         <f aca="false">E56*F56</f>
-        <v>2.5</v>
-      </c>
-      <c r="H57" s="11" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="B58" s="19"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B67" s="13"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="13"/>
+      <c r="E67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="13" t="n">
         <f aca="false">SUM(G49:G56)</f>
-        <v>29.8</v>
-      </c>
-      <c r="H58" s="14"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="21"/>
-      <c r="B59" s="21"/>
-      <c r="C59" s="21"/>
-      <c r="D59" s="21"/>
-      <c r="E59" s="21"/>
-      <c r="F59" s="21"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="B60" s="22"/>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="23" t="n">
+        <v>117.5</v>
+      </c>
+      <c r="H67" s="13"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="22"/>
+      <c r="B68" s="22"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="22"/>
+      <c r="H68" s="22"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="B69" s="23"/>
+      <c r="C69" s="23"/>
+      <c r="D69" s="23"/>
+      <c r="E69" s="23"/>
+      <c r="F69" s="23"/>
+      <c r="G69" s="23" t="n">
         <f aca="false">G10+G20+G26+G37+G47+G57</f>
-        <v>220.3</v>
-      </c>
-      <c r="H60" s="24"/>
-    </row>
-    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="B61" s="25"/>
-      <c r="C61" s="25"/>
-      <c r="D61" s="25"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="25"/>
-      <c r="G61" s="26" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H69" s="23"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="B70" s="24"/>
+      <c r="C70" s="24"/>
+      <c r="D70" s="24"/>
+      <c r="E70" s="24"/>
+      <c r="F70" s="24"/>
+      <c r="G70" s="24" t="n">
         <f aca="false">G59*0.15</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="B62" s="19"/>
-      <c r="C62" s="19"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-      <c r="F62" s="20"/>
-      <c r="G62" s="28" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H70" s="24"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="B71" s="26"/>
+      <c r="C71" s="26"/>
+      <c r="D71" s="26"/>
+      <c r="E71" s="26"/>
+      <c r="F71" s="27"/>
+      <c r="G71" s="28" t="n">
         <f aca="false">G59+G60</f>
-        <v>220.3</v>
-      </c>
-      <c r="H62" s="29"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="B64" s="30"/>
-      <c r="C64" s="30"/>
-      <c r="D64" s="30"/>
-      <c r="E64" s="30"/>
-      <c r="F64" s="30"/>
-      <c r="G64" s="30"/>
-      <c r="H64" s="30"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="B65" s="31"/>
-      <c r="C65" s="31"/>
-      <c r="D65" s="31"/>
-      <c r="E65" s="31"/>
-      <c r="F65" s="31"/>
-      <c r="G65" s="31"/>
-      <c r="H65" s="31"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="31" t="s">
-        <v>143</v>
-      </c>
-      <c r="B66" s="31"/>
-      <c r="C66" s="31"/>
-      <c r="D66" s="31"/>
-      <c r="E66" s="31"/>
-      <c r="F66" s="31"/>
-      <c r="G66" s="31"/>
-      <c r="H66" s="31"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="B67" s="31"/>
-      <c r="C67" s="31"/>
-      <c r="D67" s="31"/>
-      <c r="E67" s="31"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="31"/>
-      <c r="H67" s="31"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="31" t="s">
-        <v>145</v>
-      </c>
-      <c r="B68" s="31"/>
-      <c r="C68" s="31"/>
-      <c r="D68" s="31"/>
-      <c r="E68" s="31"/>
-      <c r="F68" s="31"/>
-      <c r="G68" s="31"/>
-      <c r="H68" s="31"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="31" t="s">
-        <v>146</v>
-      </c>
-      <c r="B69" s="31"/>
-      <c r="C69" s="31"/>
-      <c r="D69" s="31"/>
-      <c r="E69" s="31"/>
-      <c r="F69" s="31"/>
-      <c r="G69" s="31"/>
-      <c r="H69" s="31"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="31" t="s">
-        <v>147</v>
-      </c>
-      <c r="B70" s="31"/>
-      <c r="C70" s="31"/>
-      <c r="D70" s="31"/>
-      <c r="E70" s="31"/>
-      <c r="F70" s="31"/>
-      <c r="G70" s="31"/>
-      <c r="H70" s="31"/>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="32" t="s">
-        <v>148</v>
+        <v>5.5</v>
+      </c>
+      <c r="H71" s="29"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="30" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="31" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="31" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="31" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="31" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="31" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="31" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: auto-compensating drippers + per-pot chronic dryness alerts
Hydraulic:
- BOM: replaced adjustable drippers with auto-compensating (CNL) drippers
  Mix: 10× 2L/h (succulentes) + 6× 4L/h (aromates) + 4× 8L/h (tropicales)
- Constant flow regardless of tube length/position in network
- Dripper flow set once mechanically per plant type

Per-pot monitoring:
- SensorManager tracks consecutive dry readings per pot (PotAlert struct)
- After 6 consecutive readings below threshold → Telegram alert:
  '⚠ Pot #7 chroniquement sec (23%, 6 lectures) → ajuster le goutteur'
- Alert resets when pot moisture recovers above threshold
- Prevents alert spam: sent once per dry episode per pot

Philosophy: sensors monitor + alert, drippers actuate mechanically.
No electro-valves, no per-pot control — complexity stays in software, not hardware.
</commit_message>
<xml_diff>
--- a/docs/BOM_v3_plug_and_play.xlsx
+++ b/docs/BOM_v3_plug_and_play.xlsx
@@ -307,13 +307,13 @@
     <t xml:space="preserve">Rouleau 20m, alimentaire</t>
   </si>
   <si>
-    <t xml:space="preserve">Goutteurs réglables 0-70 L/h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Embase + pic, réglage individuel par plante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress (lot 20 ~8€)</t>
+    <t xml:space="preserve">Goutteurs auto-compensants (mix)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNL compensés: 10× 2L/h (succulentes) + 6× 4L/h (aromates) + 4× 8L/h (tropicales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress / Gardena (goutteurs CNL pression compensée)</t>
   </si>
   <si>
     <t xml:space="preserve">Connecteurs T / Y 4mm</t>
@@ -767,8 +767,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -784,7 +788,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -792,7 +796,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -800,11 +804,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -812,7 +816,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -820,15 +824,15 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -836,11 +840,11 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -848,7 +852,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -856,19 +860,19 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1127,1830 +1131,1830 @@
   <dimension ref="A1:H85"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="36"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="8" t="n">
+      <c r="E6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="10" t="n">
         <f aca="false">E6*F6</f>
         <v>25</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="8" t="n">
+      <c r="E7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="10" t="n">
         <f aca="false">E7*F7</f>
         <v>30</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="8" t="n">
+      <c r="E8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <f aca="false">E8*F8</f>
         <v>18</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="8" t="n">
+      <c r="E9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <f aca="false">E9*F9</f>
         <v>5</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
+    <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="8" t="n">
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="10" t="n">
         <f aca="false">E10*F10</f>
         <v>1.5</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="13" t="n">
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="14" t="n">
         <f aca="false">SUM(G6:G10)</f>
         <v>79.5</v>
       </c>
-      <c r="H11" s="14"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="H11" s="15"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="n">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="8" t="n">
+      <c r="E13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="10" t="n">
         <f aca="false">E13*F13</f>
         <v>5</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="8" t="n">
+      <c r="E14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="10" t="n">
         <f aca="false">E14*F14</f>
         <v>8</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F15" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" s="10" t="n">
         <f aca="false">E15*F15</f>
         <v>5</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="8" t="n">
+      <c r="E16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="9" t="n">
         <v>3.5</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="10" t="n">
         <f aca="false">E16*F16</f>
         <v>3.5</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="8" t="n">
+      <c r="E17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="10" t="n">
         <f aca="false">E17*F17</f>
         <v>2</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="8" t="n">
+      <c r="E18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="10" t="n">
         <f aca="false">E18*F18</f>
         <v>2</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="8" t="n">
+      <c r="E19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="9" t="n">
         <v>0.3</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G19" s="10" t="n">
         <f aca="false">E19*F19</f>
         <v>0.3</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G20" s="10" t="n">
         <f aca="false">E20*F20</f>
         <v>0.3</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G21" s="10" t="n">
         <f aca="false">E21*F21</f>
         <v>0.2</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="10" t="n">
         <f aca="false">E22*F22</f>
         <v>0.2</v>
       </c>
-      <c r="H22" s="10" t="s">
+      <c r="H22" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="9" t="n">
         <v>0.2</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G23" s="10" t="n">
         <f aca="false">E23*F23</f>
         <v>0.4</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="8" t="n">
+      <c r="E24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="9" t="n">
+      <c r="G24" s="10" t="n">
         <f aca="false">E24*F24</f>
         <v>2</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="8" t="n">
+      <c r="E25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="9" t="n">
+      <c r="G25" s="10" t="n">
         <f aca="false">E25*F25</f>
         <v>2</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="13" t="n">
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="14" t="n">
         <f aca="false">SUM(G13:G25)</f>
         <v>30.9</v>
       </c>
-      <c r="H26" s="14"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="H26" s="15"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="n">
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="F28" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="G28" s="9" t="n">
+      <c r="G28" s="10" t="n">
         <f aca="false">E28*F28</f>
         <v>16</v>
       </c>
-      <c r="H28" s="10" t="s">
+      <c r="H28" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="F29" s="9" t="n">
         <v>4.5</v>
       </c>
-      <c r="G29" s="9" t="n">
+      <c r="G29" s="10" t="n">
         <f aca="false">E29*F29</f>
         <v>9</v>
       </c>
-      <c r="H29" s="10" t="s">
+      <c r="H29" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="8" t="n">
+      <c r="E30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G30" s="9" t="n">
+      <c r="G30" s="10" t="n">
         <f aca="false">E30*F30</f>
         <v>2.5</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="8" t="n">
+      <c r="E31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G31" s="9" t="n">
+      <c r="G31" s="10" t="n">
         <f aca="false">E31*F31</f>
         <v>2.5</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="8" t="n">
+      <c r="E32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="9" t="n">
+      <c r="G32" s="10" t="n">
         <f aca="false">E32*F32</f>
         <v>2</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="H32" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="13" t="n">
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="14" t="n">
         <f aca="false">SUM(G28:G32)</f>
         <v>32</v>
       </c>
-      <c r="H33" s="14"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="H33" s="15"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="n">
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="G35" s="9" t="n">
+      <c r="G35" s="10" t="n">
         <f aca="false">E35*F35</f>
         <v>0</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="H35" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="8" t="n">
+      <c r="E36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="G36" s="9" t="n">
+      <c r="G36" s="10" t="n">
         <f aca="false">E36*F36</f>
         <v>12</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="H36" s="11" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="5" t="n">
+      <c r="E37" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F37" s="8" t="n">
+      <c r="F37" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="G37" s="9" t="n">
+      <c r="G37" s="10" t="n">
         <f aca="false">E37*F37</f>
         <v>6</v>
       </c>
-      <c r="H37" s="10" t="s">
+      <c r="H37" s="11" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="n">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="E38" s="5" t="n">
+      <c r="E38" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F38" s="8" t="n">
+      <c r="F38" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G38" s="9" t="n">
+      <c r="G38" s="10" t="n">
         <f aca="false">E38*F38</f>
         <v>6</v>
       </c>
-      <c r="H38" s="10" t="s">
+      <c r="H38" s="11" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="E39" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="8" t="n">
+      <c r="E39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G39" s="9" t="n">
+      <c r="G39" s="10" t="n">
         <f aca="false">E39*F39</f>
         <v>3</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="H39" s="11" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="E40" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G40" s="9" t="n">
+      <c r="G40" s="10" t="n">
         <f aca="false">E40*F40</f>
         <v>10</v>
       </c>
-      <c r="H40" s="10" t="s">
+      <c r="H40" s="11" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="n">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="E41" s="5" t="n">
+      <c r="E41" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F41" s="8" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G41" s="9" t="n">
+      <c r="F41" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G41" s="10" t="n">
         <f aca="false">E41*F41</f>
-        <v>8</v>
-      </c>
-      <c r="H41" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H41" s="11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="E42" s="5" t="n">
+      <c r="E42" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F42" s="9" t="n">
         <v>0.2</v>
       </c>
-      <c r="G42" s="9" t="n">
+      <c r="G42" s="10" t="n">
         <f aca="false">E42*F42</f>
         <v>4</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H42" s="11" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="n">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E43" s="5" t="n">
+      <c r="E43" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F43" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="G43" s="9" t="n">
+      <c r="G43" s="10" t="n">
         <f aca="false">E43*F43</f>
         <v>3</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="H43" s="11" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="13" t="n">
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="14" t="n">
         <f aca="false">SUM(G35:G43)</f>
-        <v>52</v>
-      </c>
-      <c r="H44" s="14"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H44" s="15"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="n">
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E46" s="5" t="n">
+      <c r="E46" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F46" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="G46" s="9" t="n">
+      <c r="G46" s="10" t="n">
         <f aca="false">E46*F46</f>
         <v>5</v>
       </c>
-      <c r="H46" s="10" t="s">
+      <c r="H46" s="11" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="n">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="D47" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="E47" s="5" t="n">
+      <c r="E47" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F47" s="8" t="n">
+      <c r="F47" s="9" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="9" t="n">
+      <c r="G47" s="10" t="n">
         <f aca="false">E47*F47</f>
         <v>6</v>
       </c>
-      <c r="H47" s="10" t="s">
+      <c r="H47" s="11" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="n">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D48" s="7" t="s">
+      <c r="D48" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="E48" s="5" t="n">
+      <c r="E48" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F48" s="8" t="n">
+      <c r="F48" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="G48" s="9" t="n">
+      <c r="G48" s="10" t="n">
         <f aca="false">E48*F48</f>
         <v>4</v>
       </c>
-      <c r="H48" s="10" t="s">
+      <c r="H48" s="11" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="n">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D49" s="7" t="s">
+      <c r="D49" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="E49" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="8" t="n">
+      <c r="E49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G49" s="9" t="n">
+      <c r="G49" s="10" t="n">
         <f aca="false">E49*F49</f>
         <v>4</v>
       </c>
-      <c r="H49" s="10" t="s">
+      <c r="H49" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="n">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="n">
         <v>37</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D50" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="E50" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="8" t="n">
+      <c r="E50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G50" s="9" t="n">
+      <c r="G50" s="10" t="n">
         <f aca="false">E50*F50</f>
         <v>3</v>
       </c>
-      <c r="H50" s="10" t="s">
+      <c r="H50" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="n">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="D51" s="7" t="s">
+      <c r="D51" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="E51" s="5" t="n">
+      <c r="E51" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="F51" s="8" t="n">
+      <c r="F51" s="9" t="n">
         <v>0.05</v>
       </c>
-      <c r="G51" s="9" t="n">
+      <c r="G51" s="10" t="n">
         <f aca="false">E51*F51</f>
         <v>2</v>
       </c>
-      <c r="H51" s="10" t="s">
+      <c r="H51" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="n">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D52" s="7" t="s">
+      <c r="D52" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="E52" s="5" t="n">
+      <c r="E52" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F52" s="8" t="n">
+      <c r="F52" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="G52" s="9" t="n">
+      <c r="G52" s="10" t="n">
         <f aca="false">E52*F52</f>
         <v>8</v>
       </c>
-      <c r="H52" s="10" t="s">
+      <c r="H52" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="n">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D53" s="7" t="s">
+      <c r="D53" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E53" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="8" t="n">
+      <c r="E53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G53" s="9" t="n">
+      <c r="G53" s="10" t="n">
         <f aca="false">E53*F53</f>
         <v>3</v>
       </c>
-      <c r="H53" s="10" t="s">
+      <c r="H53" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="5" t="n">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C54" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="D54" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="E54" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="8" t="n">
+      <c r="E54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G54" s="9" t="n">
+      <c r="G54" s="10" t="n">
         <f aca="false">E54*F54</f>
         <v>2</v>
       </c>
-      <c r="H54" s="10" t="s">
+      <c r="H54" s="11" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B55" s="12"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="12"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="13" t="n">
+      <c r="B55" s="13"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="14" t="n">
         <f aca="false">SUM(G46:G54)</f>
         <v>37</v>
       </c>
-      <c r="H55" s="14"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
+      <c r="H55" s="15"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="5" t="n">
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="D57" s="7" t="s">
+      <c r="D57" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F57" s="8" t="n">
+      <c r="E57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="G57" s="9" t="n">
+      <c r="G57" s="10" t="n">
         <f aca="false">E57*F57</f>
         <v>12</v>
       </c>
-      <c r="H57" s="10" t="s">
+      <c r="H57" s="11" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="n">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="D58" s="7" t="s">
+      <c r="D58" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E58" s="5" t="n">
+      <c r="E58" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F58" s="8" t="n">
+      <c r="F58" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="G58" s="9" t="n">
+      <c r="G58" s="10" t="n">
         <f aca="false">E58*F58</f>
         <v>4</v>
       </c>
-      <c r="H58" s="10" t="s">
+      <c r="H58" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5" t="n">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D59" s="7" t="s">
+      <c r="D59" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="E59" s="5" t="n">
+      <c r="E59" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F59" s="8" t="n">
+      <c r="F59" s="9" t="n">
         <v>0.6</v>
       </c>
-      <c r="G59" s="9" t="n">
+      <c r="G59" s="10" t="n">
         <f aca="false">E59*F59</f>
         <v>2.4</v>
       </c>
-      <c r="H59" s="10" t="s">
+      <c r="H59" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="n">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="D60" s="7" t="s">
+      <c r="D60" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="E60" s="5" t="n">
+      <c r="E60" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F60" s="8" t="n">
+      <c r="F60" s="9" t="n">
         <v>0.7</v>
       </c>
-      <c r="G60" s="9" t="n">
+      <c r="G60" s="10" t="n">
         <f aca="false">E60*F60</f>
         <v>1.4</v>
       </c>
-      <c r="H60" s="10" t="s">
+      <c r="H60" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="5" t="n">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="B61" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D61" s="7" t="s">
+      <c r="D61" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="E61" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="8" t="n">
+      <c r="E61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G61" s="9" t="n">
+      <c r="G61" s="10" t="n">
         <f aca="false">E61*F61</f>
         <v>2.5</v>
       </c>
-      <c r="H61" s="10" t="s">
+      <c r="H61" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="n">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B62" s="6" t="s">
+      <c r="B62" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C62" s="6" t="s">
+      <c r="C62" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D62" s="7" t="s">
+      <c r="D62" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="E62" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F62" s="8" t="n">
+      <c r="E62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G62" s="9" t="n">
+      <c r="G62" s="10" t="n">
         <f aca="false">E62*F62</f>
         <v>2</v>
       </c>
-      <c r="H62" s="10" t="s">
+      <c r="H62" s="11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5" t="n">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="B63" s="6" t="s">
+      <c r="B63" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C63" s="6" t="s">
+      <c r="C63" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="D63" s="7" t="s">
+      <c r="D63" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="E63" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F63" s="8" t="n">
+      <c r="E63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G63" s="9" t="n">
+      <c r="G63" s="10" t="n">
         <f aca="false">E63*F63</f>
         <v>3</v>
       </c>
-      <c r="H63" s="10" t="s">
+      <c r="H63" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="5" t="n">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B64" s="6" t="s">
+      <c r="B64" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C64" s="6" t="s">
+      <c r="C64" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="D64" s="7" t="s">
+      <c r="D64" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="E64" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F64" s="8" t="n">
+      <c r="E64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>2.5</v>
       </c>
-      <c r="G64" s="9" t="n">
+      <c r="G64" s="10" t="n">
         <f aca="false">E64*F64</f>
         <v>2.5</v>
       </c>
-      <c r="H64" s="10" t="s">
+      <c r="H64" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="12" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B65" s="12"/>
-      <c r="C65" s="12"/>
-      <c r="D65" s="12"/>
-      <c r="E65" s="12"/>
-      <c r="F65" s="12"/>
-      <c r="G65" s="13" t="n">
+      <c r="B65" s="13"/>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
+      <c r="E65" s="13"/>
+      <c r="F65" s="13"/>
+      <c r="G65" s="14" t="n">
         <f aca="false">SUM(G57:G64)</f>
         <v>29.8</v>
       </c>
-      <c r="H65" s="14"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="4" t="s">
+      <c r="H65" s="15"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="B66" s="4"/>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="5" t="n">
+      <c r="B66" s="5"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B67" s="6" t="s">
+      <c r="B67" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="C67" s="6" t="s">
+      <c r="C67" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="D67" s="7" t="s">
+      <c r="D67" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="E67" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" s="8" t="n">
+      <c r="E67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="G67" s="9" t="n">
+      <c r="G67" s="10" t="n">
         <f aca="false">E67*F67</f>
         <v>15</v>
       </c>
-      <c r="H67" s="10" t="s">
+      <c r="H67" s="11" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="5" t="n">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="B68" s="6" t="s">
+      <c r="B68" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="C68" s="6" t="s">
+      <c r="C68" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="D68" s="7" t="s">
+      <c r="D68" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="E68" s="5" t="n">
+      <c r="E68" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F68" s="8" t="n">
+      <c r="F68" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="G68" s="9" t="n">
+      <c r="G68" s="10" t="n">
         <f aca="false">E68*F68</f>
         <v>6</v>
       </c>
-      <c r="H68" s="10" t="s">
+      <c r="H68" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="n">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="B69" s="6" t="s">
+      <c r="B69" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="C69" s="6" t="s">
+      <c r="C69" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="D69" s="7" t="s">
+      <c r="D69" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="E69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" s="8" t="n">
+      <c r="E69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G69" s="9" t="n">
+      <c r="G69" s="10" t="n">
         <f aca="false">E69*F69</f>
         <v>3</v>
       </c>
-      <c r="H69" s="10" t="s">
+      <c r="H69" s="11" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="5" t="n">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="6" t="n">
         <v>53</v>
       </c>
-      <c r="B70" s="6" t="s">
+      <c r="B70" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="C70" s="6" t="s">
+      <c r="C70" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D70" s="7" t="s">
+      <c r="D70" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="E70" s="5" t="n">
+      <c r="E70" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F70" s="8" t="n">
+      <c r="F70" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G70" s="9" t="n">
+      <c r="G70" s="10" t="n">
         <f aca="false">E70*F70</f>
         <v>6</v>
       </c>
-      <c r="H70" s="10" t="s">
+      <c r="H70" s="11" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="12" t="s">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="B71" s="12"/>
-      <c r="C71" s="12"/>
-      <c r="D71" s="12"/>
-      <c r="E71" s="12"/>
-      <c r="F71" s="12"/>
-      <c r="G71" s="13" t="n">
+      <c r="B71" s="13"/>
+      <c r="C71" s="13"/>
+      <c r="D71" s="13"/>
+      <c r="E71" s="13"/>
+      <c r="F71" s="13"/>
+      <c r="G71" s="14" t="n">
         <f aca="false">SUM(G67:G70)</f>
         <v>30</v>
       </c>
-      <c r="H71" s="14"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="16" t="s">
+      <c r="H71" s="15"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="B73" s="16"/>
-      <c r="C73" s="16"/>
-      <c r="D73" s="16"/>
-      <c r="E73" s="16"/>
-      <c r="F73" s="16"/>
-      <c r="G73" s="17" t="n">
+      <c r="B73" s="17"/>
+      <c r="C73" s="17"/>
+      <c r="D73" s="17"/>
+      <c r="E73" s="17"/>
+      <c r="F73" s="17"/>
+      <c r="G73" s="18" t="n">
         <f aca="false">G11+G26+G33+G44+G55+G65+G71</f>
-        <v>291.2</v>
-      </c>
-      <c r="H73" s="18"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="19" t="s">
+        <v>293.2</v>
+      </c>
+      <c r="H73" s="19"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="B74" s="19"/>
-      <c r="C74" s="19"/>
-      <c r="D74" s="19"/>
-      <c r="E74" s="19"/>
-      <c r="F74" s="19"/>
-      <c r="G74" s="20" t="n">
+      <c r="B74" s="20"/>
+      <c r="C74" s="20"/>
+      <c r="D74" s="20"/>
+      <c r="E74" s="20"/>
+      <c r="F74" s="20"/>
+      <c r="G74" s="21" t="n">
         <f aca="false">G73*0.15</f>
-        <v>43.68</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="21" t="s">
+        <v>43.98</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B75" s="21"/>
-      <c r="C75" s="21"/>
-      <c r="D75" s="21"/>
-      <c r="E75" s="21"/>
-      <c r="F75" s="21"/>
-      <c r="G75" s="22" t="n">
+      <c r="B75" s="22"/>
+      <c r="C75" s="22"/>
+      <c r="D75" s="22"/>
+      <c r="E75" s="22"/>
+      <c r="F75" s="22"/>
+      <c r="G75" s="23" t="n">
         <f aca="false">G73+G74</f>
-        <v>334.88</v>
-      </c>
-      <c r="H75" s="23"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="24" t="s">
+        <v>337.18</v>
+      </c>
+      <c r="H75" s="24"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="25" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="25" t="s">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="B78" s="25"/>
-      <c r="C78" s="25"/>
-      <c r="D78" s="25"/>
-      <c r="E78" s="25"/>
-      <c r="F78" s="25"/>
-      <c r="G78" s="25"/>
-      <c r="H78" s="25"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="25" t="s">
+      <c r="B78" s="26"/>
+      <c r="C78" s="26"/>
+      <c r="D78" s="26"/>
+      <c r="E78" s="26"/>
+      <c r="F78" s="26"/>
+      <c r="G78" s="26"/>
+      <c r="H78" s="26"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="26" t="s">
         <v>167</v>
       </c>
-      <c r="B79" s="25"/>
-      <c r="C79" s="25"/>
-      <c r="D79" s="25"/>
-      <c r="E79" s="25"/>
-      <c r="F79" s="25"/>
-      <c r="G79" s="25"/>
-      <c r="H79" s="25"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="25" t="s">
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
+      <c r="F79" s="26"/>
+      <c r="G79" s="26"/>
+      <c r="H79" s="26"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="B80" s="25"/>
-      <c r="C80" s="25"/>
-      <c r="D80" s="25"/>
-      <c r="E80" s="25"/>
-      <c r="F80" s="25"/>
-      <c r="G80" s="25"/>
-      <c r="H80" s="25"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="25" t="s">
+      <c r="B80" s="26"/>
+      <c r="C80" s="26"/>
+      <c r="D80" s="26"/>
+      <c r="E80" s="26"/>
+      <c r="F80" s="26"/>
+      <c r="G80" s="26"/>
+      <c r="H80" s="26"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="26" t="s">
         <v>169</v>
       </c>
-      <c r="B81" s="25"/>
-      <c r="C81" s="25"/>
-      <c r="D81" s="25"/>
-      <c r="E81" s="25"/>
-      <c r="F81" s="25"/>
-      <c r="G81" s="25"/>
-      <c r="H81" s="25"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="25" t="s">
+      <c r="B81" s="26"/>
+      <c r="C81" s="26"/>
+      <c r="D81" s="26"/>
+      <c r="E81" s="26"/>
+      <c r="F81" s="26"/>
+      <c r="G81" s="26"/>
+      <c r="H81" s="26"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="B82" s="25"/>
-      <c r="C82" s="25"/>
-      <c r="D82" s="25"/>
-      <c r="E82" s="25"/>
-      <c r="F82" s="25"/>
-      <c r="G82" s="25"/>
-      <c r="H82" s="25"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="25" t="s">
+      <c r="B82" s="26"/>
+      <c r="C82" s="26"/>
+      <c r="D82" s="26"/>
+      <c r="E82" s="26"/>
+      <c r="F82" s="26"/>
+      <c r="G82" s="26"/>
+      <c r="H82" s="26"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="26" t="s">
         <v>171</v>
       </c>
-      <c r="B83" s="25"/>
-      <c r="C83" s="25"/>
-      <c r="D83" s="25"/>
-      <c r="E83" s="25"/>
-      <c r="F83" s="25"/>
-      <c r="G83" s="25"/>
-      <c r="H83" s="25"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="25" t="s">
+      <c r="B83" s="26"/>
+      <c r="C83" s="26"/>
+      <c r="D83" s="26"/>
+      <c r="E83" s="26"/>
+      <c r="F83" s="26"/>
+      <c r="G83" s="26"/>
+      <c r="H83" s="26"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="26" t="s">
         <v>172</v>
       </c>
-      <c r="B84" s="25"/>
-      <c r="C84" s="25"/>
-      <c r="D84" s="25"/>
-      <c r="E84" s="25"/>
-      <c r="F84" s="25"/>
-      <c r="G84" s="25"/>
-      <c r="H84" s="25"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="25" t="s">
+      <c r="B84" s="26"/>
+      <c r="C84" s="26"/>
+      <c r="D84" s="26"/>
+      <c r="E84" s="26"/>
+      <c r="F84" s="26"/>
+      <c r="G84" s="26"/>
+      <c r="H84" s="26"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="B85" s="25"/>
-      <c r="C85" s="25"/>
-      <c r="D85" s="25"/>
-      <c r="E85" s="25"/>
-      <c r="F85" s="25"/>
-      <c r="G85" s="25"/>
-      <c r="H85" s="25"/>
+      <c r="B85" s="26"/>
+      <c r="C85" s="26"/>
+      <c r="D85" s="26"/>
+      <c r="E85" s="26"/>
+      <c r="F85" s="26"/>
+      <c r="G85" s="26"/>
+      <c r="H85" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>